<commit_message>
Update crop_estimates.xlsx with TCH and Area
</commit_message>
<xml_diff>
--- a/data/crop_estimates.xlsx
+++ b/data/crop_estimates.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="81">
   <si>
     <t>Date</t>
   </si>
@@ -256,14 +256,21 @@
   </si>
   <si>
     <t>168.80</t>
+  </si>
+  <si>
+    <t>Area (ha)</t>
+  </si>
+  <si>
+    <t>TCH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -314,12 +321,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,13 +631,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:M103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -639,16 +649,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>45376</v>
       </c>
@@ -658,14 +674,21 @@
       <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3">
+        <v>19.686</v>
+      </c>
+      <c r="E2" s="4">
+        <v>95</v>
+      </c>
+      <c r="F2">
         <v>1870.17</v>
       </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="4"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45376</v>
       </c>
@@ -675,14 +698,21 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="3">
+        <v>9.1349999999999998</v>
+      </c>
+      <c r="E3" s="4">
+        <v>70</v>
+      </c>
+      <c r="F3">
         <v>639.44999999999993</v>
       </c>
-      <c r="F3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M3" s="4"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45376</v>
       </c>
@@ -692,14 +722,21 @@
       <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="3">
+        <v>11.3</v>
+      </c>
+      <c r="E4" s="4">
+        <v>82</v>
+      </c>
+      <c r="F4">
         <v>926.6</v>
       </c>
-      <c r="F4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>8</v>
+      </c>
+      <c r="M4" s="4"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45376</v>
       </c>
@@ -709,14 +746,21 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="3">
+        <v>16.341999999999999</v>
+      </c>
+      <c r="E5" s="4">
+        <v>34.08701505323706</v>
+      </c>
+      <c r="F5">
         <v>557.04999999999995</v>
       </c>
-      <c r="F5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>8</v>
+      </c>
+      <c r="M5" s="4"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45376</v>
       </c>
@@ -726,14 +770,21 @@
       <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="3">
+        <v>17.327999999999999</v>
+      </c>
+      <c r="E6" s="4">
+        <v>85.000000000000014</v>
+      </c>
+      <c r="F6">
         <v>1472.88</v>
       </c>
-      <c r="F6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>8</v>
+      </c>
+      <c r="M6" s="4"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45376</v>
       </c>
@@ -743,14 +794,21 @@
       <c r="C7" t="s">
         <v>12</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="3">
+        <v>15.696999999999999</v>
+      </c>
+      <c r="E7" s="4">
+        <v>93.438555137924439</v>
+      </c>
+      <c r="F7">
         <v>1466.7049999999999</v>
       </c>
-      <c r="F7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>8</v>
+      </c>
+      <c r="M7" s="4"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45376</v>
       </c>
@@ -760,14 +818,21 @@
       <c r="C8" t="s">
         <v>18</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="3">
+        <v>19.280999999999999</v>
+      </c>
+      <c r="E8" s="4">
+        <v>84.529329391629062</v>
+      </c>
+      <c r="F8">
         <v>1629.81</v>
       </c>
-      <c r="F8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" s="4"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45376</v>
       </c>
@@ -777,14 +842,21 @@
       <c r="C9" t="s">
         <v>12</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="3">
+        <v>17.605</v>
+      </c>
+      <c r="E9" s="4">
+        <v>77.814257313263283</v>
+      </c>
+      <c r="F9">
         <v>1369.92</v>
       </c>
-      <c r="F9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>8</v>
+      </c>
+      <c r="M9" s="4"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45376</v>
       </c>
@@ -794,14 +866,21 @@
       <c r="C10" t="s">
         <v>10</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="3">
+        <v>31.706</v>
+      </c>
+      <c r="E10" s="4">
+        <v>75</v>
+      </c>
+      <c r="F10">
         <v>2377.9499999999998</v>
       </c>
-      <c r="F10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>8</v>
+      </c>
+      <c r="M10" s="4"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45376</v>
       </c>
@@ -811,14 +890,21 @@
       <c r="C11" t="s">
         <v>7</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="3">
+        <v>21.465</v>
+      </c>
+      <c r="E11" s="4">
+        <v>70</v>
+      </c>
+      <c r="F11">
         <v>1502.55</v>
       </c>
-      <c r="F11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>8</v>
+      </c>
+      <c r="M11" s="4"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>45376</v>
       </c>
@@ -828,14 +914,21 @@
       <c r="C12" t="s">
         <v>23</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="3">
+        <v>42.033000000000001</v>
+      </c>
+      <c r="E12" s="4">
+        <v>90.000000000000028</v>
+      </c>
+      <c r="F12">
         <v>3782.9700000000012</v>
       </c>
-      <c r="F12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>8</v>
+      </c>
+      <c r="M12" s="4"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45376</v>
       </c>
@@ -845,14 +938,21 @@
       <c r="C13" t="s">
         <v>7</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="3">
+        <v>23.658000000000001</v>
+      </c>
+      <c r="E13" s="4">
+        <v>74.999999999999986</v>
+      </c>
+      <c r="F13">
         <v>1774.35</v>
       </c>
-      <c r="F13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>8</v>
+      </c>
+      <c r="M13" s="4"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>45376</v>
       </c>
@@ -862,14 +962,21 @@
       <c r="C14" t="s">
         <v>12</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="3">
+        <v>35.624000000000002</v>
+      </c>
+      <c r="E14" s="4">
+        <v>92.407927240062875</v>
+      </c>
+      <c r="F14">
         <v>3291.94</v>
       </c>
-      <c r="F14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>8</v>
+      </c>
+      <c r="M14" s="4"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>45376</v>
       </c>
@@ -879,14 +986,21 @@
       <c r="C15" t="s">
         <v>12</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="3">
+        <v>14.504</v>
+      </c>
+      <c r="E15" s="4">
+        <v>50.000000000000007</v>
+      </c>
+      <c r="F15">
         <v>725.2</v>
       </c>
-      <c r="F15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>8</v>
+      </c>
+      <c r="M15" s="4"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45376</v>
       </c>
@@ -896,14 +1010,21 @@
       <c r="C16" t="s">
         <v>10</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="3">
+        <v>25.122</v>
+      </c>
+      <c r="E16" s="4">
+        <v>13.888225459756388</v>
+      </c>
+      <c r="F16">
         <v>348.9</v>
       </c>
-      <c r="F16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>8</v>
+      </c>
+      <c r="M16" s="4"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>45376</v>
       </c>
@@ -913,14 +1034,21 @@
       <c r="C17" t="s">
         <v>18</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="3">
+        <v>4.1950000000000003</v>
+      </c>
+      <c r="E17" s="4">
+        <v>84.999999999999986</v>
+      </c>
+      <c r="F17">
         <v>356.57499999999999</v>
       </c>
-      <c r="F17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>8</v>
+      </c>
+      <c r="M17" s="4"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>45376</v>
       </c>
@@ -930,14 +1058,21 @@
       <c r="C18" t="s">
         <v>14</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="3">
+        <v>16.079000000000001</v>
+      </c>
+      <c r="E18" s="4">
+        <v>60</v>
+      </c>
+      <c r="F18">
         <v>964.74</v>
       </c>
-      <c r="F18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>8</v>
+      </c>
+      <c r="M18" s="4"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>45376</v>
       </c>
@@ -947,14 +1082,21 @@
       <c r="C19" t="s">
         <v>14</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="3">
+        <v>14.065</v>
+      </c>
+      <c r="E19" s="4">
+        <v>90</v>
+      </c>
+      <c r="F19">
         <v>1265.8499999999999</v>
       </c>
-      <c r="F19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>8</v>
+      </c>
+      <c r="M19" s="4"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>45376</v>
       </c>
@@ -964,14 +1106,21 @@
       <c r="C20" t="s">
         <v>12</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="3">
+        <v>16.888999999999999</v>
+      </c>
+      <c r="E20" s="4">
+        <v>70</v>
+      </c>
+      <c r="F20">
         <v>1182.23</v>
       </c>
-      <c r="F20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>8</v>
+      </c>
+      <c r="M20" s="4"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>45376</v>
       </c>
@@ -981,14 +1130,21 @@
       <c r="C21" t="s">
         <v>10</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="3">
+        <v>23.146999999999998</v>
+      </c>
+      <c r="E21" s="4">
+        <v>70</v>
+      </c>
+      <c r="F21">
         <v>1620.29</v>
       </c>
-      <c r="F21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>8</v>
+      </c>
+      <c r="M21" s="4"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45376</v>
       </c>
@@ -998,14 +1154,21 @@
       <c r="C22" t="s">
         <v>12</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="3">
+        <v>18.552</v>
+      </c>
+      <c r="E22" s="4">
+        <v>59.999999999999993</v>
+      </c>
+      <c r="F22">
         <v>1113.1199999999999</v>
       </c>
-      <c r="F22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>8</v>
+      </c>
+      <c r="M22" s="4"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45376</v>
       </c>
@@ -1015,14 +1178,21 @@
       <c r="C23" t="s">
         <v>14</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="3">
+        <v>24.803999999999998</v>
+      </c>
+      <c r="E23" s="4">
+        <v>90.000000000000014</v>
+      </c>
+      <c r="F23">
         <v>2232.36</v>
       </c>
-      <c r="F23" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>8</v>
+      </c>
+      <c r="M23" s="4"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45376</v>
       </c>
@@ -1032,14 +1202,21 @@
       <c r="C24" t="s">
         <v>12</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="3">
+        <v>19.149999999999999</v>
+      </c>
+      <c r="E24" s="4">
+        <v>55.000000000000007</v>
+      </c>
+      <c r="F24">
         <v>1053.25</v>
       </c>
-      <c r="F24" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>8</v>
+      </c>
+      <c r="M24" s="4"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45376</v>
       </c>
@@ -1049,14 +1226,21 @@
       <c r="C25" t="s">
         <v>14</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="3">
+        <v>25.193000000000001</v>
+      </c>
+      <c r="E25" s="4">
+        <v>81.626046917794625</v>
+      </c>
+      <c r="F25">
         <v>2056.4050000000002</v>
       </c>
-      <c r="F25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>8</v>
+      </c>
+      <c r="M25" s="4"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45376</v>
       </c>
@@ -1066,14 +1250,21 @@
       <c r="C26" t="s">
         <v>12</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="3">
+        <v>18.324999999999999</v>
+      </c>
+      <c r="E26" s="4">
+        <v>80</v>
+      </c>
+      <c r="F26">
         <v>1466</v>
       </c>
-      <c r="F26" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>8</v>
+      </c>
+      <c r="M26" s="4"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45376</v>
       </c>
@@ -1083,14 +1274,21 @@
       <c r="C27" t="s">
         <v>10</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="3">
+        <v>24.106999999999999</v>
+      </c>
+      <c r="E27" s="4">
+        <v>75</v>
+      </c>
+      <c r="F27">
         <v>1808.0250000000001</v>
       </c>
-      <c r="F27" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>8</v>
+      </c>
+      <c r="M27" s="4"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45376</v>
       </c>
@@ -1100,14 +1298,21 @@
       <c r="C28" t="s">
         <v>14</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="3">
+        <v>13.993</v>
+      </c>
+      <c r="E28" s="4">
+        <v>89.999999999999986</v>
+      </c>
+      <c r="F28">
         <v>1259.3699999999999</v>
       </c>
-      <c r="F28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H28" t="s">
+        <v>8</v>
+      </c>
+      <c r="M28" s="4"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45376</v>
       </c>
@@ -1117,14 +1322,21 @@
       <c r="C29" t="s">
         <v>12</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="3">
+        <v>23.161999999999999</v>
+      </c>
+      <c r="E29" s="4">
+        <v>50</v>
+      </c>
+      <c r="F29">
         <v>1158.0999999999999</v>
       </c>
-      <c r="F29" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H29" t="s">
+        <v>8</v>
+      </c>
+      <c r="M29" s="4"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45376</v>
       </c>
@@ -1134,14 +1346,21 @@
       <c r="C30" t="s">
         <v>12</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="3">
+        <v>8.423</v>
+      </c>
+      <c r="E30" s="4">
+        <v>95.139498990858371</v>
+      </c>
+      <c r="F30">
         <v>801.36</v>
       </c>
-      <c r="F30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H30" t="s">
+        <v>8</v>
+      </c>
+      <c r="M30" s="4"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45376</v>
       </c>
@@ -1151,14 +1370,21 @@
       <c r="C31" t="s">
         <v>12</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="3">
+        <v>21.858000000000001</v>
+      </c>
+      <c r="E31" s="4">
+        <v>43.043736846921036</v>
+      </c>
+      <c r="F31">
         <v>940.85</v>
       </c>
-      <c r="F31" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>8</v>
+      </c>
+      <c r="M31" s="4"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45376</v>
       </c>
@@ -1168,14 +1394,21 @@
       <c r="C32" t="s">
         <v>14</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="3">
+        <v>25.047000000000001</v>
+      </c>
+      <c r="E32" s="4">
+        <v>90</v>
+      </c>
+      <c r="F32">
         <v>2254.23</v>
       </c>
-      <c r="F32" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>8</v>
+      </c>
+      <c r="M32" s="4"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45376</v>
       </c>
@@ -1185,14 +1418,21 @@
       <c r="C33" t="s">
         <v>14</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="3">
+        <v>21.138000000000002</v>
+      </c>
+      <c r="E33" s="4">
+        <v>70</v>
+      </c>
+      <c r="F33">
         <v>1479.66</v>
       </c>
-      <c r="F33" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H33" t="s">
+        <v>8</v>
+      </c>
+      <c r="M33" s="4"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45376</v>
       </c>
@@ -1202,14 +1442,21 @@
       <c r="C34" t="s">
         <v>10</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="3">
+        <v>24.542999999999999</v>
+      </c>
+      <c r="E34" s="4">
+        <v>80</v>
+      </c>
+      <c r="F34">
         <v>1963.44</v>
       </c>
-      <c r="F34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H34" t="s">
+        <v>8</v>
+      </c>
+      <c r="M34" s="4"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45376</v>
       </c>
@@ -1219,14 +1466,21 @@
       <c r="C35" t="s">
         <v>14</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="3">
+        <v>12.795999999999999</v>
+      </c>
+      <c r="E35" s="4">
+        <v>78.780869021569245</v>
+      </c>
+      <c r="F35">
         <v>1008.08</v>
       </c>
-      <c r="F35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M35" s="4"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45376</v>
       </c>
@@ -1236,14 +1490,21 @@
       <c r="C36" t="s">
         <v>12</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="3">
+        <v>9.7799999999999994</v>
+      </c>
+      <c r="E36" s="4">
+        <v>60</v>
+      </c>
+      <c r="F36">
         <v>586.79999999999995</v>
       </c>
-      <c r="F36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H36" t="s">
+        <v>8</v>
+      </c>
+      <c r="M36" s="4"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45376</v>
       </c>
@@ -1253,14 +1514,21 @@
       <c r="C37" t="s">
         <v>10</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="3">
+        <v>11.125</v>
+      </c>
+      <c r="E37" s="4">
+        <v>80</v>
+      </c>
+      <c r="F37">
         <v>890</v>
       </c>
-      <c r="F37" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H37" t="s">
+        <v>8</v>
+      </c>
+      <c r="M37" s="4"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45376</v>
       </c>
@@ -1270,14 +1538,21 @@
       <c r="C38" t="s">
         <v>10</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="3">
+        <v>10.439</v>
+      </c>
+      <c r="E38" s="4">
+        <v>90</v>
+      </c>
+      <c r="F38">
         <v>939.51</v>
       </c>
-      <c r="F38" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>8</v>
+      </c>
+      <c r="M38" s="4"/>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45376</v>
       </c>
@@ -1287,14 +1562,21 @@
       <c r="C39" t="s">
         <v>10</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="3">
+        <v>7.1740000000000004</v>
+      </c>
+      <c r="E39" s="4">
+        <v>89.999999999999986</v>
+      </c>
+      <c r="F39">
         <v>645.66</v>
       </c>
-      <c r="F39" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H39" t="s">
+        <v>8</v>
+      </c>
+      <c r="M39" s="4"/>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45376</v>
       </c>
@@ -1304,14 +1586,21 @@
       <c r="C40" t="s">
         <v>12</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="3">
+        <v>8.7379999999999995</v>
+      </c>
+      <c r="E40" s="4">
+        <v>65</v>
+      </c>
+      <c r="F40">
         <v>567.97</v>
       </c>
-      <c r="F40" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H40" t="s">
+        <v>8</v>
+      </c>
+      <c r="M40" s="4"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45376</v>
       </c>
@@ -1321,14 +1610,21 @@
       <c r="C41" t="s">
         <v>14</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="3">
+        <v>13.321</v>
+      </c>
+      <c r="E41" s="4">
+        <v>54.999999999999993</v>
+      </c>
+      <c r="F41">
         <v>732.65499999999986</v>
       </c>
-      <c r="F41" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H41" t="s">
+        <v>8</v>
+      </c>
+      <c r="M41" s="4"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45376</v>
       </c>
@@ -1338,14 +1634,21 @@
       <c r="C42" t="s">
         <v>12</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="3">
+        <v>18.931000000000001</v>
+      </c>
+      <c r="E42" s="4">
+        <v>45</v>
+      </c>
+      <c r="F42">
         <v>851.8950000000001</v>
       </c>
-      <c r="F42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H42" t="s">
+        <v>8</v>
+      </c>
+      <c r="M42" s="4"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45376</v>
       </c>
@@ -1355,14 +1658,21 @@
       <c r="C43" t="s">
         <v>14</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="3">
         <v>0</v>
       </c>
-      <c r="F43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E43" s="4">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="H43" t="s">
+        <v>8</v>
+      </c>
+      <c r="M43" s="4"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45376</v>
       </c>
@@ -1372,14 +1682,21 @@
       <c r="C44" t="s">
         <v>14</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="3">
+        <v>25.213999999999999</v>
+      </c>
+      <c r="E44" s="4">
+        <v>35.339097326881884</v>
+      </c>
+      <c r="F44">
         <v>891.03999999999985</v>
       </c>
-      <c r="F44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H44" t="s">
+        <v>8</v>
+      </c>
+      <c r="M44" s="4"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45376</v>
       </c>
@@ -1389,14 +1706,21 @@
       <c r="C45" t="s">
         <v>14</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="3">
+        <v>7.4450000000000003</v>
+      </c>
+      <c r="E45" s="4">
+        <v>44.999999999999993</v>
+      </c>
+      <c r="F45">
         <v>335.02499999999998</v>
       </c>
-      <c r="F45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H45" t="s">
+        <v>8</v>
+      </c>
+      <c r="M45" s="4"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45376</v>
       </c>
@@ -1406,14 +1730,21 @@
       <c r="C46" t="s">
         <v>14</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="3">
+        <v>1.27</v>
+      </c>
+      <c r="E46" s="4">
+        <v>56.480314960629926</v>
+      </c>
+      <c r="F46">
         <v>71.73</v>
       </c>
-      <c r="F46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H46" t="s">
+        <v>8</v>
+      </c>
+      <c r="M46" s="4"/>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45376</v>
       </c>
@@ -1423,28 +1754,42 @@
       <c r="C47" t="s">
         <v>14</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="3">
+        <v>2.8849999999999998</v>
+      </c>
+      <c r="E47" s="4">
+        <v>30</v>
+      </c>
+      <c r="F47">
         <v>86.55</v>
       </c>
-      <c r="F47" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H47" t="s">
+        <v>8</v>
+      </c>
+      <c r="M47" s="4"/>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45376</v>
       </c>
       <c r="B48" t="s">
         <v>59</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="3">
         <v>0</v>
       </c>
-      <c r="F48" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E48" s="4">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="H48" t="s">
+        <v>8</v>
+      </c>
+      <c r="M48" s="4"/>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45376</v>
       </c>
@@ -1454,14 +1799,21 @@
       <c r="C49" t="s">
         <v>14</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="3">
+        <v>15.798</v>
+      </c>
+      <c r="E49" s="4">
+        <v>34.538549183440942</v>
+      </c>
+      <c r="F49">
         <v>545.64</v>
       </c>
-      <c r="F49" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H49" t="s">
+        <v>8</v>
+      </c>
+      <c r="M49" s="4"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45376</v>
       </c>
@@ -1471,14 +1823,21 @@
       <c r="C50" t="s">
         <v>14</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="3">
+        <v>5.3449999999999998</v>
+      </c>
+      <c r="E50" s="4">
+        <v>24.658559401309638</v>
+      </c>
+      <c r="F50">
         <v>131.80000000000001</v>
       </c>
-      <c r="F50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H50" t="s">
+        <v>8</v>
+      </c>
+      <c r="M50" s="4"/>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45376</v>
       </c>
@@ -1488,28 +1847,42 @@
       <c r="C51" t="s">
         <v>12</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="3">
+        <v>4.0940000000000003</v>
+      </c>
+      <c r="E51" s="4">
+        <v>47.936003908158277</v>
+      </c>
+      <c r="F51">
         <v>196.25</v>
       </c>
-      <c r="F51" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H51" t="s">
+        <v>8</v>
+      </c>
+      <c r="M51" s="4"/>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45376</v>
       </c>
       <c r="B52" t="s">
         <v>63</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="3">
         <v>0</v>
       </c>
-      <c r="F52" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E52" s="4">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="H52" t="s">
+        <v>8</v>
+      </c>
+      <c r="M52" s="4"/>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45376</v>
       </c>
@@ -1519,14 +1892,21 @@
       <c r="C53" t="s">
         <v>12</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="3">
+        <v>3.07</v>
+      </c>
+      <c r="E53" s="4">
+        <v>48.371335504885998</v>
+      </c>
+      <c r="F53">
         <v>148.5</v>
       </c>
-      <c r="F53" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H53" t="s">
+        <v>8</v>
+      </c>
+      <c r="M53" s="4"/>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45736</v>
       </c>
@@ -1536,17 +1916,24 @@
       <c r="C54" t="s">
         <v>7</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="3">
+        <v>19.686</v>
+      </c>
+      <c r="E54" s="4">
+        <v>105.00000000000001</v>
+      </c>
+      <c r="F54">
         <v>2067.0300000000002</v>
       </c>
-      <c r="E54" t="s">
+      <c r="G54" t="s">
         <v>65</v>
       </c>
-      <c r="F54" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H54" t="s">
+        <v>66</v>
+      </c>
+      <c r="M54" s="4"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45736</v>
       </c>
@@ -1556,17 +1943,24 @@
       <c r="C55" t="s">
         <v>18</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="3">
+        <v>9.1349999999999998</v>
+      </c>
+      <c r="E55" s="4">
+        <v>88</v>
+      </c>
+      <c r="F55">
         <v>803.88</v>
       </c>
-      <c r="E55" t="s">
+      <c r="G55" t="s">
         <v>67</v>
       </c>
-      <c r="F55" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H55" t="s">
+        <v>66</v>
+      </c>
+      <c r="M55" s="4"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45736</v>
       </c>
@@ -1576,17 +1970,24 @@
       <c r="C56" t="s">
         <v>12</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="3">
+        <v>11.3</v>
+      </c>
+      <c r="E56" s="4">
+        <v>89.899999999999991</v>
+      </c>
+      <c r="F56">
         <v>1015.87</v>
       </c>
-      <c r="E56" t="s">
+      <c r="G56" t="s">
         <v>68</v>
       </c>
-      <c r="F56" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H56" t="s">
+        <v>66</v>
+      </c>
+      <c r="M56" s="4"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45736</v>
       </c>
@@ -1596,17 +1997,24 @@
       <c r="C57" t="s">
         <v>14</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="3">
+        <v>10.141</v>
+      </c>
+      <c r="E57" s="4">
+        <v>89.925056700522632</v>
+      </c>
+      <c r="F57">
         <v>911.93</v>
       </c>
-      <c r="E57" t="s">
+      <c r="G57" t="s">
         <v>69</v>
       </c>
-      <c r="F57" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H57" t="s">
+        <v>66</v>
+      </c>
+      <c r="M57" s="4"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45736</v>
       </c>
@@ -1616,17 +2024,24 @@
       <c r="C58" t="s">
         <v>10</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="3">
+        <v>17.327999999999999</v>
+      </c>
+      <c r="E58" s="4">
+        <v>96.000115420129276</v>
+      </c>
+      <c r="F58">
         <v>1663.49</v>
       </c>
-      <c r="E58" t="s">
+      <c r="G58" t="s">
         <v>65</v>
       </c>
-      <c r="F58" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H58" t="s">
+        <v>66</v>
+      </c>
+      <c r="M58" s="4"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>70</v>
       </c>
@@ -1636,14 +2051,21 @@
       <c r="C59" t="s">
         <v>12</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="3">
+        <v>15.439</v>
+      </c>
+      <c r="E59" s="4">
+        <v>97.999870457931209</v>
+      </c>
+      <c r="F59">
         <v>1513.02</v>
       </c>
-      <c r="F59" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H59" t="s">
+        <v>66</v>
+      </c>
+      <c r="M59" s="4"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>70</v>
       </c>
@@ -1653,17 +2075,24 @@
       <c r="C60" t="s">
         <v>18</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="3">
+        <v>18.895</v>
+      </c>
+      <c r="E60" s="4">
+        <v>90</v>
+      </c>
+      <c r="F60">
         <v>1700.55</v>
       </c>
-      <c r="E60" t="s">
+      <c r="G60" t="s">
         <v>71</v>
       </c>
-      <c r="F60" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H60" t="s">
+        <v>66</v>
+      </c>
+      <c r="M60" s="4"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>70</v>
       </c>
@@ -1673,14 +2102,21 @@
       <c r="C61" t="s">
         <v>12</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="3">
+        <v>17.123999999999999</v>
+      </c>
+      <c r="E61" s="4">
+        <v>90.000000000000014</v>
+      </c>
+      <c r="F61">
         <v>1541.16</v>
       </c>
-      <c r="F61" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H61" t="s">
+        <v>66</v>
+      </c>
+      <c r="M61" s="4"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -1690,14 +2126,21 @@
       <c r="C62" t="s">
         <v>10</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="3">
+        <v>31.706</v>
+      </c>
+      <c r="E62" s="4">
+        <v>90</v>
+      </c>
+      <c r="F62">
         <v>2853.54</v>
       </c>
-      <c r="F62" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H62" t="s">
+        <v>66</v>
+      </c>
+      <c r="M62" s="4"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>70</v>
       </c>
@@ -1707,14 +2150,21 @@
       <c r="C63" t="s">
         <v>7</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="3">
+        <v>21.465</v>
+      </c>
+      <c r="E63" s="4">
+        <v>85.00023293733986</v>
+      </c>
+      <c r="F63">
         <v>1824.53</v>
       </c>
-      <c r="F63" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H63" t="s">
+        <v>66</v>
+      </c>
+      <c r="M63" s="4"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>70</v>
       </c>
@@ -1724,14 +2174,21 @@
       <c r="C64" t="s">
         <v>23</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="3">
+        <v>42.033000000000001</v>
+      </c>
+      <c r="E64" s="4">
+        <v>105.00011895415507</v>
+      </c>
+      <c r="F64">
         <v>4413.47</v>
       </c>
-      <c r="F64" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H64" t="s">
+        <v>66</v>
+      </c>
+      <c r="M64" s="4"/>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>70</v>
       </c>
@@ -1741,14 +2198,21 @@
       <c r="C65" t="s">
         <v>7</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="3">
+        <v>23.658000000000001</v>
+      </c>
+      <c r="E65" s="4">
+        <v>80</v>
+      </c>
+      <c r="F65">
         <v>1892.64</v>
       </c>
-      <c r="F65" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H65" t="s">
+        <v>66</v>
+      </c>
+      <c r="M65" s="4"/>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>70</v>
       </c>
@@ -1758,17 +2222,24 @@
       <c r="C66" t="s">
         <v>12</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="3">
+        <v>34.652000000000001</v>
+      </c>
+      <c r="E66" s="4">
+        <v>99.999999999999986</v>
+      </c>
+      <c r="F66">
         <v>3465.2</v>
       </c>
-      <c r="E66" t="s">
+      <c r="G66" t="s">
         <v>71</v>
       </c>
-      <c r="F66" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H66" t="s">
+        <v>66</v>
+      </c>
+      <c r="M66" s="4"/>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>70</v>
       </c>
@@ -1778,14 +2249,21 @@
       <c r="C67" t="s">
         <v>12</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="3">
+        <v>14.504</v>
+      </c>
+      <c r="E67" s="4">
+        <v>62.000137892995035</v>
+      </c>
+      <c r="F67">
         <v>899.25</v>
       </c>
-      <c r="F67" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H67" t="s">
+        <v>66</v>
+      </c>
+      <c r="M67" s="4"/>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>70</v>
       </c>
@@ -1795,17 +2273,24 @@
       <c r="C68" t="s">
         <v>10</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="3">
+        <v>25.122</v>
+      </c>
+      <c r="E68" s="4">
+        <v>65</v>
+      </c>
+      <c r="F68">
         <v>1632.93</v>
       </c>
-      <c r="E68" t="s">
+      <c r="G68" t="s">
         <v>71</v>
       </c>
-      <c r="F68" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H68" t="s">
+        <v>66</v>
+      </c>
+      <c r="M68" s="4"/>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>70</v>
       </c>
@@ -1815,17 +2300,24 @@
       <c r="C69" t="s">
         <v>18</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="3">
+        <v>4.1950000000000003</v>
+      </c>
+      <c r="E69" s="4">
+        <v>111.99999999999999</v>
+      </c>
+      <c r="F69">
         <v>469.84</v>
       </c>
-      <c r="E69" t="s">
+      <c r="G69" t="s">
         <v>71</v>
       </c>
-      <c r="F69" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H69" t="s">
+        <v>66</v>
+      </c>
+      <c r="M69" s="4"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>70</v>
       </c>
@@ -1835,14 +2327,21 @@
       <c r="C70" t="s">
         <v>14</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="3">
+        <v>16.079000000000001</v>
+      </c>
+      <c r="E70" s="4">
+        <v>50</v>
+      </c>
+      <c r="F70">
         <v>803.95</v>
       </c>
-      <c r="F70" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H70" t="s">
+        <v>66</v>
+      </c>
+      <c r="M70" s="4"/>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -1852,14 +2351,21 @@
       <c r="C71" t="s">
         <v>12</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="3">
+        <v>14.065</v>
+      </c>
+      <c r="E71" s="4">
+        <v>95.000355492356917</v>
+      </c>
+      <c r="F71">
         <v>1336.18</v>
       </c>
-      <c r="F71" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H71" t="s">
+        <v>66</v>
+      </c>
+      <c r="M71" s="4"/>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>70</v>
       </c>
@@ -1869,14 +2375,21 @@
       <c r="C72" t="s">
         <v>12</v>
       </c>
-      <c r="D72">
+      <c r="D72" s="3">
+        <v>16.888999999999999</v>
+      </c>
+      <c r="E72" s="4">
+        <v>70</v>
+      </c>
+      <c r="F72">
         <v>1182.23</v>
       </c>
-      <c r="F72" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H72" t="s">
+        <v>66</v>
+      </c>
+      <c r="M72" s="4"/>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -1886,17 +2399,24 @@
       <c r="C73" t="s">
         <v>12</v>
       </c>
-      <c r="D73">
+      <c r="D73" s="3">
+        <v>23.146999999999998</v>
+      </c>
+      <c r="E73" s="4">
+        <v>58.560072579599954</v>
+      </c>
+      <c r="F73">
         <v>1355.49</v>
       </c>
-      <c r="E73" t="s">
+      <c r="G73" t="s">
         <v>73</v>
       </c>
-      <c r="F73" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H73" t="s">
+        <v>66</v>
+      </c>
+      <c r="M73" s="4"/>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>72</v>
       </c>
@@ -1906,14 +2426,21 @@
       <c r="C74" t="s">
         <v>14</v>
       </c>
-      <c r="D74">
+      <c r="D74" s="3">
+        <v>18.552</v>
+      </c>
+      <c r="E74" s="4">
+        <v>50</v>
+      </c>
+      <c r="F74">
         <v>927.6</v>
       </c>
-      <c r="F74" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H74" t="s">
+        <v>66</v>
+      </c>
+      <c r="M74" s="4"/>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>72</v>
       </c>
@@ -1923,14 +2450,21 @@
       <c r="C75" t="s">
         <v>14</v>
       </c>
-      <c r="D75">
+      <c r="D75" s="3">
+        <v>24.803999999999998</v>
+      </c>
+      <c r="E75" s="4">
+        <v>82.000080632156113</v>
+      </c>
+      <c r="F75">
         <v>2033.93</v>
       </c>
-      <c r="F75" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H75" t="s">
+        <v>66</v>
+      </c>
+      <c r="M75" s="4"/>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>72</v>
       </c>
@@ -1940,14 +2474,21 @@
       <c r="C76" t="s">
         <v>12</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="3">
+        <v>19.149999999999999</v>
+      </c>
+      <c r="E76" s="4">
+        <v>50.000000000000007</v>
+      </c>
+      <c r="F76">
         <v>957.5</v>
       </c>
-      <c r="F76" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H76" t="s">
+        <v>66</v>
+      </c>
+      <c r="M76" s="4"/>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>72</v>
       </c>
@@ -1957,14 +2498,21 @@
       <c r="C77" t="s">
         <v>7</v>
       </c>
-      <c r="D77">
+      <c r="D77" s="3">
+        <v>25.193000000000001</v>
+      </c>
+      <c r="E77" s="4">
+        <v>80</v>
+      </c>
+      <c r="F77">
         <v>2015.44</v>
       </c>
-      <c r="F77" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H77" t="s">
+        <v>66</v>
+      </c>
+      <c r="M77" s="4"/>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>72</v>
       </c>
@@ -1974,14 +2522,21 @@
       <c r="C78" t="s">
         <v>12</v>
       </c>
-      <c r="D78">
+      <c r="D78" s="3">
+        <v>18.324999999999999</v>
+      </c>
+      <c r="E78" s="4">
+        <v>70</v>
+      </c>
+      <c r="F78">
         <v>1282.75</v>
       </c>
-      <c r="F78" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H78" t="s">
+        <v>66</v>
+      </c>
+      <c r="M78" s="4"/>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>72</v>
       </c>
@@ -1991,14 +2546,21 @@
       <c r="C79" t="s">
         <v>10</v>
       </c>
-      <c r="D79">
+      <c r="D79" s="3">
+        <v>24.106999999999999</v>
+      </c>
+      <c r="E79" s="4">
+        <v>70</v>
+      </c>
+      <c r="F79">
         <v>1687.49</v>
       </c>
-      <c r="F79" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H79" t="s">
+        <v>66</v>
+      </c>
+      <c r="M79" s="4"/>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>72</v>
       </c>
@@ -2008,17 +2570,24 @@
       <c r="C80" t="s">
         <v>14</v>
       </c>
-      <c r="D80">
+      <c r="D80" s="3">
+        <v>13.993</v>
+      </c>
+      <c r="E80" s="4">
+        <v>86.999928535696426</v>
+      </c>
+      <c r="F80">
         <v>1217.3900000000001</v>
       </c>
-      <c r="E80" t="s">
+      <c r="G80" t="s">
         <v>74</v>
       </c>
-      <c r="F80" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H80" t="s">
+        <v>66</v>
+      </c>
+      <c r="M80" s="4"/>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>72</v>
       </c>
@@ -2028,17 +2597,24 @@
       <c r="C81" t="s">
         <v>12</v>
       </c>
-      <c r="D81">
+      <c r="D81" s="3">
+        <v>23.161999999999999</v>
+      </c>
+      <c r="E81" s="4">
+        <v>80</v>
+      </c>
+      <c r="F81">
         <v>1852.96</v>
       </c>
-      <c r="E81" t="s">
+      <c r="G81" t="s">
         <v>73</v>
       </c>
-      <c r="F81" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H81" t="s">
+        <v>66</v>
+      </c>
+      <c r="M81" s="4"/>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>72</v>
       </c>
@@ -2048,14 +2624,21 @@
       <c r="C82" t="s">
         <v>12</v>
       </c>
-      <c r="D82">
+      <c r="D82" s="3">
+        <v>8.9039999999999999</v>
+      </c>
+      <c r="E82" s="4">
+        <v>100</v>
+      </c>
+      <c r="F82">
         <v>890.4</v>
       </c>
-      <c r="F82" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H82" t="s">
+        <v>66</v>
+      </c>
+      <c r="M82" s="4"/>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>72</v>
       </c>
@@ -2065,17 +2648,24 @@
       <c r="C83" t="s">
         <v>12</v>
       </c>
-      <c r="D83">
+      <c r="D83" s="3">
+        <v>21.858000000000001</v>
+      </c>
+      <c r="E83" s="4">
+        <v>70</v>
+      </c>
+      <c r="F83">
         <v>1530.06</v>
       </c>
-      <c r="E83" t="s">
+      <c r="G83" t="s">
         <v>71</v>
       </c>
-      <c r="F83" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H83" t="s">
+        <v>66</v>
+      </c>
+      <c r="M83" s="4"/>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>72</v>
       </c>
@@ -2085,14 +2675,21 @@
       <c r="C84" t="s">
         <v>14</v>
       </c>
-      <c r="D84">
+      <c r="D84" s="3">
+        <v>25.047000000000001</v>
+      </c>
+      <c r="E84" s="4">
+        <v>90</v>
+      </c>
+      <c r="F84">
         <v>2254.23</v>
       </c>
-      <c r="F84" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H84" t="s">
+        <v>66</v>
+      </c>
+      <c r="M84" s="4"/>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>72</v>
       </c>
@@ -2102,14 +2699,21 @@
       <c r="C85" t="s">
         <v>14</v>
       </c>
-      <c r="D85">
+      <c r="D85" s="3">
+        <v>21.138000000000002</v>
+      </c>
+      <c r="E85" s="4">
+        <v>85</v>
+      </c>
+      <c r="F85">
         <v>1796.73</v>
       </c>
-      <c r="F85" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H85" t="s">
+        <v>66</v>
+      </c>
+      <c r="M85" s="4"/>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>72</v>
       </c>
@@ -2119,14 +2723,21 @@
       <c r="C86" t="s">
         <v>10</v>
       </c>
-      <c r="D86">
+      <c r="D86" s="3">
+        <v>24.542999999999999</v>
+      </c>
+      <c r="E86" s="4">
+        <v>80</v>
+      </c>
+      <c r="F86">
         <v>1963.44</v>
       </c>
-      <c r="F86" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H86" t="s">
+        <v>66</v>
+      </c>
+      <c r="M86" s="4"/>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>72</v>
       </c>
@@ -2136,17 +2747,24 @@
       <c r="C87" t="s">
         <v>18</v>
       </c>
-      <c r="D87">
+      <c r="D87" s="3">
+        <v>12.601000000000001</v>
+      </c>
+      <c r="E87" s="4">
+        <v>90.160304737719215</v>
+      </c>
+      <c r="F87">
         <v>1136.1099999999999</v>
       </c>
-      <c r="E87" t="s">
+      <c r="G87" t="s">
         <v>73</v>
       </c>
-      <c r="F87" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H87" t="s">
+        <v>66</v>
+      </c>
+      <c r="M87" s="4"/>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>72</v>
       </c>
@@ -2156,17 +2774,24 @@
       <c r="C88" t="s">
         <v>12</v>
       </c>
-      <c r="D88">
+      <c r="D88" s="3">
+        <v>9.7799999999999994</v>
+      </c>
+      <c r="E88" s="4">
+        <v>70</v>
+      </c>
+      <c r="F88">
         <v>684.6</v>
       </c>
-      <c r="E88" t="s">
+      <c r="G88" t="s">
         <v>75</v>
       </c>
-      <c r="F88" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H88" t="s">
+        <v>66</v>
+      </c>
+      <c r="M88" s="4"/>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>72</v>
       </c>
@@ -2176,17 +2801,24 @@
       <c r="C89" t="s">
         <v>10</v>
       </c>
-      <c r="D89">
+      <c r="D89" s="3">
+        <v>11.125</v>
+      </c>
+      <c r="E89" s="4">
+        <v>79.900224719101118</v>
+      </c>
+      <c r="F89">
         <v>888.89</v>
       </c>
-      <c r="E89" t="s">
+      <c r="G89" t="s">
         <v>75</v>
       </c>
-      <c r="F89" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H89" t="s">
+        <v>66</v>
+      </c>
+      <c r="M89" s="4"/>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>72</v>
       </c>
@@ -2196,14 +2828,21 @@
       <c r="C90" t="s">
         <v>10</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="3">
+        <v>10.439</v>
+      </c>
+      <c r="E90" s="4">
+        <v>100.00000000000001</v>
+      </c>
+      <c r="F90">
         <v>1043.9000000000001</v>
       </c>
-      <c r="F90" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H90" t="s">
+        <v>66</v>
+      </c>
+      <c r="M90" s="4"/>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>72</v>
       </c>
@@ -2213,14 +2852,21 @@
       <c r="C91" t="s">
         <v>10</v>
       </c>
-      <c r="D91">
+      <c r="D91" s="3">
+        <v>7.1740000000000004</v>
+      </c>
+      <c r="E91" s="4">
+        <v>99.999999999999986</v>
+      </c>
+      <c r="F91">
         <v>717.4</v>
       </c>
-      <c r="F91" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H91" t="s">
+        <v>66</v>
+      </c>
+      <c r="M91" s="4"/>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>72</v>
       </c>
@@ -2230,17 +2876,24 @@
       <c r="C92" t="s">
         <v>12</v>
       </c>
-      <c r="D92">
+      <c r="D92" s="3">
+        <v>8.7379999999999995</v>
+      </c>
+      <c r="E92" s="4">
+        <v>50</v>
+      </c>
+      <c r="F92">
         <v>436.9</v>
       </c>
-      <c r="E92" t="s">
+      <c r="G92" t="s">
         <v>74</v>
       </c>
-      <c r="F92" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H92" t="s">
+        <v>66</v>
+      </c>
+      <c r="M92" s="4"/>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>72</v>
       </c>
@@ -2250,14 +2903,21 @@
       <c r="C93" t="s">
         <v>14</v>
       </c>
-      <c r="D93">
+      <c r="D93" s="3">
+        <v>13.321</v>
+      </c>
+      <c r="E93" s="4">
+        <v>60</v>
+      </c>
+      <c r="F93">
         <v>799.26</v>
       </c>
-      <c r="F93" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H93" t="s">
+        <v>66</v>
+      </c>
+      <c r="M93" s="4"/>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>72</v>
       </c>
@@ -2267,17 +2927,24 @@
       <c r="C94" t="s">
         <v>12</v>
       </c>
-      <c r="D94">
+      <c r="D94" s="3">
+        <v>13.906000000000001</v>
+      </c>
+      <c r="E94" s="4">
+        <v>30</v>
+      </c>
+      <c r="F94">
         <v>417.18</v>
       </c>
-      <c r="E94" t="s">
+      <c r="G94" t="s">
         <v>76</v>
       </c>
-      <c r="F94" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H94" t="s">
+        <v>66</v>
+      </c>
+      <c r="M94" s="4"/>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>72</v>
       </c>
@@ -2287,17 +2954,24 @@
       <c r="C95" t="s">
         <v>14</v>
       </c>
-      <c r="D95">
+      <c r="D95" s="3">
+        <v>2.4460000000000002</v>
+      </c>
+      <c r="E95" s="4">
+        <v>40</v>
+      </c>
+      <c r="F95">
         <v>97.84</v>
       </c>
-      <c r="E95" t="s">
+      <c r="G95" t="s">
         <v>73</v>
       </c>
-      <c r="F95" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H95" t="s">
+        <v>66</v>
+      </c>
+      <c r="M95" s="4"/>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>72</v>
       </c>
@@ -2307,17 +2981,24 @@
       <c r="C96" t="s">
         <v>14</v>
       </c>
-      <c r="D96">
+      <c r="D96" s="3">
+        <v>8.907</v>
+      </c>
+      <c r="E96" s="4">
+        <v>25.00056135623667</v>
+      </c>
+      <c r="F96">
         <v>222.68</v>
       </c>
-      <c r="E96" t="s">
+      <c r="G96" t="s">
         <v>76</v>
       </c>
-      <c r="F96" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H96" t="s">
+        <v>66</v>
+      </c>
+      <c r="M96" s="4"/>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>72</v>
       </c>
@@ -2327,14 +3008,21 @@
       <c r="C97" t="s">
         <v>14</v>
       </c>
-      <c r="D97">
+      <c r="D97" s="3">
+        <v>7.4450000000000003</v>
+      </c>
+      <c r="E97" s="4">
+        <v>35.000671591672258</v>
+      </c>
+      <c r="F97">
         <v>260.58</v>
       </c>
-      <c r="F97" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H97" t="s">
+        <v>66</v>
+      </c>
+      <c r="M97" s="4"/>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>72</v>
       </c>
@@ -2344,17 +3032,24 @@
       <c r="C98" t="s">
         <v>14</v>
       </c>
-      <c r="D98">
+      <c r="D98" s="3">
+        <v>1.27</v>
+      </c>
+      <c r="E98" s="4">
+        <v>65.897637795275585</v>
+      </c>
+      <c r="F98">
         <v>83.69</v>
       </c>
-      <c r="E98" t="s">
+      <c r="G98" t="s">
         <v>77</v>
       </c>
-      <c r="F98" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H98" t="s">
+        <v>66</v>
+      </c>
+      <c r="M98" s="4"/>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>72</v>
       </c>
@@ -2364,14 +3059,21 @@
       <c r="C99" t="s">
         <v>14</v>
       </c>
-      <c r="D99">
+      <c r="D99" s="3">
+        <v>2.8849999999999998</v>
+      </c>
+      <c r="E99" s="4">
+        <v>45.001733102253041</v>
+      </c>
+      <c r="F99">
         <v>129.83000000000001</v>
       </c>
-      <c r="F99" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H99" t="s">
+        <v>66</v>
+      </c>
+      <c r="M99" s="4"/>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>72</v>
       </c>
@@ -2381,14 +3083,21 @@
       <c r="C100" t="s">
         <v>14</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="3">
+        <v>18.957999999999998</v>
+      </c>
+      <c r="E100" s="4">
+        <v>25</v>
+      </c>
+      <c r="F100">
         <v>473.95</v>
       </c>
-      <c r="F100" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H100" t="s">
+        <v>66</v>
+      </c>
+      <c r="M100" s="4"/>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>72</v>
       </c>
@@ -2398,14 +3107,21 @@
       <c r="C101" t="s">
         <v>14</v>
       </c>
-      <c r="D101">
+      <c r="D101" s="3">
+        <v>1.9119999999999999</v>
+      </c>
+      <c r="E101" s="4">
+        <v>25</v>
+      </c>
+      <c r="F101">
         <v>47.8</v>
       </c>
-      <c r="F101" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H101" t="s">
+        <v>66</v>
+      </c>
+      <c r="M101" s="4"/>
+    </row>
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>72</v>
       </c>
@@ -2415,14 +3131,21 @@
       <c r="C102" t="s">
         <v>7</v>
       </c>
-      <c r="D102">
+      <c r="D102" s="3">
+        <v>3.9249999999999998</v>
+      </c>
+      <c r="E102" s="4">
+        <v>55.001273885350322</v>
+      </c>
+      <c r="F102">
         <v>215.88</v>
       </c>
-      <c r="F102" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H102" t="s">
+        <v>66</v>
+      </c>
+      <c r="M102" s="4"/>
+    </row>
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>72</v>
       </c>
@@ -2432,12 +3155,19 @@
       <c r="C103" t="s">
         <v>7</v>
       </c>
-      <c r="D103" t="s">
+      <c r="D103" s="3">
+        <v>3.069</v>
+      </c>
+      <c r="E103" s="4">
+        <v>55.001629195177586</v>
+      </c>
+      <c r="F103" t="s">
         <v>78</v>
       </c>
-      <c r="F103" t="s">
-        <v>66</v>
-      </c>
+      <c r="H103" t="s">
+        <v>66</v>
+      </c>
+      <c r="M103" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>